<commit_message>
updated 12V fan to stronger version, alternative link to fischer cooler
</commit_message>
<xml_diff>
--- a/hardware/uven2-mk3.xlsx
+++ b/hardware/uven2-mk3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\letrend\Documents\UVen\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7E1D8E-F429-490B-9418-D5C26AD6A48B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20DFB1F6-C74D-4C04-981C-F5F1C0423991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -140,12 +140,6 @@
     <t>https://www.digikey.de/en/products/detail/e-switch/E200-R22-C10R/24614866</t>
   </si>
   <si>
-    <t>Adafruit AHT20 - Temperature &amp; Humidity Sensor Breakout Board</t>
-  </si>
-  <si>
-    <t>https://eckstein-shop.de/AdafruitAHT20-Temperature26HumiditySensorBreakoutBoardEN</t>
-  </si>
-  <si>
     <t>GEN4-ULCD-24DT</t>
   </si>
   <si>
@@ -155,9 +149,6 @@
     <t>HA60151V4-1000U-A99</t>
   </si>
   <si>
-    <t>https://www.digikey.de/en/products/detail/sunon-fans/HA60151V4-1000U-A99/6198730</t>
-  </si>
-  <si>
     <t>Power Plug</t>
   </si>
   <si>
@@ -471,6 +462,15 @@
   </si>
   <si>
     <t>shipping costs+customs</t>
+  </si>
+  <si>
+    <t>https://de.farnell.com/en-DE/fischer-elektronik/la-v-30-150-12/k-hlk-rper-l-fter-70-m3-h-12-vdc/dp/4708578?srsltid=AfmBOopHEAoj-rLFzaWQwLiyDVg3We92MJk7J_Sfz4go-pZkLUPG5o0y</t>
+  </si>
+  <si>
+    <t>alternative</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/en/products/detail/sunon-fans/MF60151VX-1000U-A99/6198740</t>
   </si>
 </sst>
 </file>
@@ -478,8 +478,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="_-* #,##0.00&quot; €&quot;_-;\-* #,##0.00&quot; €&quot;_-;_-* \-??&quot; €&quot;_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_-[$€-2]\ * #,##0.00_-;\-[$€-2]\ * #,##0.00_-;_-[$€-2]\ * \-??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00&quot; €&quot;_-;\-* #,##0.00&quot; €&quot;_-;_-* \-??&quot; €&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-[$€-2]\ * #,##0.00_-;\-[$€-2]\ * #,##0.00_-;_-[$€-2]\ * \-??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -530,19 +530,19 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -879,15 +879,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
     <col min="2" max="2" width="16.28515625" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="5" max="5" width="143.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -898,10 +899,13 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -912,12 +916,12 @@
         <v>19.43</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -926,10 +930,10 @@
         <v>4.13</v>
       </c>
       <c r="E3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -940,10 +944,10 @@
         <v>38.520000000000003</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -954,10 +958,10 @@
         <v>29.15</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -968,10 +972,10 @@
         <v>18.43</v>
       </c>
       <c r="E6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -982,12 +986,12 @@
         <v>28.84</v>
       </c>
       <c r="E7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -996,10 +1000,10 @@
         <v>8.0399999999999991</v>
       </c>
       <c r="E8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1010,10 +1014,10 @@
         <v>0.84</v>
       </c>
       <c r="E9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1024,12 +1028,12 @@
         <v>8.66</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1038,10 +1042,10 @@
         <v>0.86</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1052,10 +1056,10 @@
         <v>25.59</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1066,10 +1070,10 @@
         <v>38.520000000000003</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1080,12 +1084,12 @@
         <v>20.53</v>
       </c>
       <c r="E14" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1094,10 +1098,10 @@
         <v>0.86</v>
       </c>
       <c r="E15" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1109,7 +1113,7 @@
         <v>52.56</v>
       </c>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1123,7 +1127,7 @@
         <v>17.71</v>
       </c>
       <c r="E17" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1137,7 +1141,7 @@
         <v>7.71</v>
       </c>
       <c r="E18" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1151,12 +1155,12 @@
         <v>0.86</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1165,7 +1169,7 @@
         <v>2.5499999999999998</v>
       </c>
       <c r="E20" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1179,7 +1183,7 @@
         <v>0.86</v>
       </c>
       <c r="E21" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1193,7 +1197,7 @@
         <v>36.18</v>
       </c>
       <c r="E22" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1207,7 +1211,7 @@
         <v>6.89</v>
       </c>
       <c r="E23" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1221,7 +1225,7 @@
         <v>10.41</v>
       </c>
       <c r="E24" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1236,7 +1240,7 @@
         <v>1.72</v>
       </c>
       <c r="E25" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1250,12 +1254,12 @@
         <v>36.18</v>
       </c>
       <c r="E26" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -1264,7 +1268,7 @@
         <v>11.86</v>
       </c>
       <c r="E27" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1278,7 +1282,7 @@
         <v>8.8800000000000008</v>
       </c>
       <c r="E28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1292,7 +1296,7 @@
         <v>5.96</v>
       </c>
       <c r="E29" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1306,7 +1310,7 @@
         <v>27.07</v>
       </c>
       <c r="E30" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1320,12 +1324,12 @@
         <v>44.98</v>
       </c>
       <c r="E31" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B32">
         <v>1</v>
@@ -1334,12 +1338,12 @@
         <v>0.86</v>
       </c>
       <c r="E32" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B33">
         <v>2</v>
@@ -1348,10 +1352,10 @@
         <v>8.66</v>
       </c>
       <c r="E33" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -1362,12 +1366,12 @@
         <v>48.86</v>
       </c>
       <c r="E34" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B35">
         <v>1</v>
@@ -1376,10 +1380,10 @@
         <v>0.86</v>
       </c>
       <c r="E35" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -1390,12 +1394,12 @@
         <v>0.86</v>
       </c>
       <c r="E36" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B37">
         <v>1</v>
@@ -1404,10 +1408,10 @@
         <v>8.8800000000000008</v>
       </c>
       <c r="E37" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>31</v>
       </c>
@@ -1419,10 +1423,10 @@
         <v>3.04</v>
       </c>
       <c r="E38" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -1433,10 +1437,10 @@
         <v>0.86</v>
       </c>
       <c r="E39" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -1447,18 +1451,18 @@
         <v>0.86</v>
       </c>
       <c r="E40" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C41" s="6">
         <v>300</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>32</v>
       </c>
@@ -1472,176 +1476,178 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>34</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" s="1">
-        <f>5.95*B43</f>
-        <v>11.9</v>
+        <v>38.619999999999997</v>
       </c>
       <c r="E43" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>36</v>
       </c>
       <c r="B44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C44" s="1">
-        <v>38.619999999999997</v>
+        <f>6.84*B44</f>
+        <v>27.36</v>
       </c>
       <c r="E44" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1">
+        <v>27.25</v>
+      </c>
+      <c r="E45" t="s">
         <v>38</v>
       </c>
-      <c r="B45">
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46">
         <v>4</v>
       </c>
-      <c r="C45" s="1">
-        <f>4.42*B45</f>
-        <v>17.68</v>
-      </c>
-      <c r="E45" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="C46" s="1">
+        <f>81.27*B46</f>
+        <v>325.08</v>
+      </c>
+      <c r="E46" t="s">
         <v>40</v>
       </c>
-      <c r="B46">
-        <v>1</v>
-      </c>
-      <c r="C46" s="1">
-        <v>27.25</v>
-      </c>
-      <c r="E46" t="s">
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" s="1">
+        <v>387.69</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B47">
-        <v>4</v>
-      </c>
-      <c r="C47" s="1">
-        <f>81.27*B47</f>
-        <v>325.08</v>
-      </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>44</v>
-      </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" s="1">
-        <v>387.69</v>
+        <v>104.92</v>
       </c>
       <c r="E48" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C49" s="1">
-        <v>104.92</v>
+        <v>334.91</v>
       </c>
       <c r="E49" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B50">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C50" s="1">
-        <v>334.91</v>
+        <v>78.260000000000005</v>
       </c>
       <c r="E50" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B51">
         <v>1</v>
       </c>
       <c r="C51" s="1">
-        <v>78.260000000000005</v>
+        <v>76.11</v>
       </c>
       <c r="E51" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>47</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" s="6">
+        <v>109.71</v>
+      </c>
+      <c r="E52" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B53">
+        <v>99</v>
+      </c>
+      <c r="C53" s="6">
+        <f>8.74*B53</f>
+        <v>865.26</v>
+      </c>
+      <c r="E53" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B52">
-        <v>1</v>
-      </c>
-      <c r="C52" s="1">
-        <v>76.11</v>
-      </c>
-      <c r="E52" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>50</v>
       </c>
-      <c r="B53">
-        <v>1</v>
-      </c>
-      <c r="C53" s="6">
-        <v>109.71</v>
-      </c>
-      <c r="E53" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" s="1">
+        <v>36.47</v>
+      </c>
+      <c r="E54" t="s">
         <v>51</v>
-      </c>
-      <c r="B54">
-        <v>100</v>
-      </c>
-      <c r="C54" s="6">
-        <f>8.74*B54</f>
-        <v>874</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1649,10 +1655,10 @@
         <v>53</v>
       </c>
       <c r="B55">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C55" s="1">
-        <v>36.47</v>
+        <v>6.07</v>
       </c>
       <c r="E55" t="s">
         <v>54</v>
@@ -1660,101 +1666,101 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B56">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C56" s="1">
-        <v>6.07</v>
+        <v>6.66</v>
       </c>
       <c r="E56" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B57">
-        <v>22</v>
+        <v>350</v>
       </c>
       <c r="C57" s="1">
-        <v>6.66</v>
-      </c>
-      <c r="E57" t="s">
-        <v>57</v>
+        <v>9.08</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B58">
-        <v>350</v>
+        <v>6</v>
       </c>
       <c r="C58" s="1">
-        <v>9.08</v>
-      </c>
-      <c r="E58" s="4" t="s">
-        <v>78</v>
+        <v>8.6300000000000008</v>
+      </c>
+      <c r="E58" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B59">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C59" s="1">
-        <v>8.6300000000000008</v>
+        <v>10.99</v>
       </c>
       <c r="E59" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>60</v>
+      </c>
+      <c r="B60">
+        <v>8</v>
+      </c>
+      <c r="C60" s="1">
+        <v>7.99</v>
+      </c>
+      <c r="E60" t="s">
         <v>61</v>
-      </c>
-      <c r="B60">
-        <v>4</v>
-      </c>
-      <c r="C60" s="1">
-        <v>10.99</v>
-      </c>
-      <c r="E60" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>62</v>
+      </c>
+      <c r="B61">
+        <v>2</v>
+      </c>
+      <c r="C61" s="1">
+        <f>1.05*B61</f>
+        <v>2.1</v>
+      </c>
+      <c r="E61" t="s">
         <v>63</v>
-      </c>
-      <c r="B61">
-        <v>8</v>
-      </c>
-      <c r="C61" s="1">
-        <v>7.99</v>
-      </c>
-      <c r="E61" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62">
+        <v>12</v>
+      </c>
+      <c r="C62" s="1">
+        <v>11.31</v>
+      </c>
+      <c r="E62" t="s">
         <v>65</v>
-      </c>
-      <c r="B62">
-        <v>2</v>
-      </c>
-      <c r="C62" s="1">
-        <f>1.05*B62</f>
-        <v>2.1</v>
-      </c>
-      <c r="E62" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1762,24 +1768,24 @@
         <v>67</v>
       </c>
       <c r="B63">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C63" s="1">
-        <v>11.31</v>
+        <v>8.59</v>
       </c>
       <c r="E63" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B64">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C64" s="1">
-        <v>8.59</v>
+        <v>3.78</v>
       </c>
       <c r="E64" t="s">
         <v>69</v>
@@ -1787,86 +1793,86 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B65">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C65" s="1">
-        <v>3.78</v>
+        <v>7.84</v>
       </c>
       <c r="E65" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B66">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C66" s="1">
-        <v>7.84</v>
+        <v>9.8800000000000008</v>
       </c>
       <c r="E66" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B67">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C67" s="1">
-        <v>9.8800000000000008</v>
+        <v>5.33</v>
       </c>
       <c r="E67" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B68">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C68" s="1">
-        <v>5.33</v>
+        <v>7</v>
       </c>
       <c r="E68" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B69">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C69" s="1">
-        <v>7</v>
+        <v>32.64</v>
       </c>
       <c r="E69" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" s="1">
-        <v>32.64</v>
+        <v>17.32</v>
       </c>
       <c r="E70" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -1874,41 +1880,41 @@
         <v>79</v>
       </c>
       <c r="B71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" s="1">
-        <v>17.32</v>
+        <v>1.19</v>
       </c>
       <c r="E71" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B72">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="C72" s="1">
-        <v>1.19</v>
+        <v>0.1</v>
       </c>
       <c r="E72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B73">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C73" s="1">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="E73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -1916,38 +1922,25 @@
         <v>86</v>
       </c>
       <c r="B74">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C74" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="E74" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>89</v>
-      </c>
-      <c r="B75">
-        <v>1</v>
-      </c>
-      <c r="C75" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C80" s="3">
-        <f>SUM(C2:C79)</f>
-        <v>3521.6000000000004</v>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C79" s="3">
+        <f>SUM(C2:C78)</f>
+        <v>3510.6400000000008</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E58" r:id="rId1" xr:uid="{FFA81BDA-DD74-4D64-A280-914C50CBA945}"/>
-    <hyperlink ref="E54" r:id="rId2" xr:uid="{D802E364-6A6E-4536-B3D3-A5BC67583CD7}"/>
+    <hyperlink ref="E57" r:id="rId1" xr:uid="{FFA81BDA-DD74-4D64-A280-914C50CBA945}"/>
+    <hyperlink ref="E53" r:id="rId2" xr:uid="{D802E364-6A6E-4536-B3D3-A5BC67583CD7}"/>
+    <hyperlink ref="E47" r:id="rId3" xr:uid="{2BAA2678-47EC-412D-A04B-CC518D24A6AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>